<commit_message>
Initial commit: Seguimiento de Contrataciones v1.1.6 - Estado actual de desarrollo
- Sistema completo de seguimiento de procesos de contratación POA 2026
- 227 procesos, 11.3K etapas, base de datos normalizada
- Backend: Node.js/Express con API REST completa
- Frontend: Vue 3 con Vite
- Autenticación por directiones y roles granulares
- Sistema de notificaciones por correo
- Auditoría completa de cambios
- Chat IA integrado con Ollama
- Migraciones de base de datos incluidas
</commit_message>
<xml_diff>
--- a/Documentos base/Empleado.xlsx
+++ b/Documentos base/Empleado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://quitoturismo365-my.sharepoint.com/personal/acasa_quito-turismo_gob_ec/Documents/Documentos/Desarrollo/Seguimiento_contrataciones/Documentos base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_CDCE3CC62AC92ABE180E5B60751BF013512D7B47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0305CA46-45FF-4AC9-AD34-7CC6FC37CBC3}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_CDCE3CC62AC92ABE180E5B60751BF013512D7B47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DF7AAB0-B5DC-4964-8207-FBF457ED623C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39540" yWindow="1140" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -908,14 +908,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:C81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="30.7109375" customWidth="1"/>
+    <col min="1" max="3" width="30.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -926,7 +925,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -937,7 +936,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -948,7 +947,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -959,7 +958,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -970,7 +969,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -981,7 +980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
@@ -992,7 +991,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1003,7 +1002,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -1014,7 +1013,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1025,7 +1024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -1036,7 +1035,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -1047,7 +1046,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -1058,7 +1057,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -1069,7 +1068,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -1080,7 +1079,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>38</v>
       </c>
@@ -1091,7 +1090,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>40</v>
       </c>
@@ -1102,7 +1101,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>43</v>
       </c>
@@ -1111,7 +1110,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>45</v>
       </c>
@@ -1122,7 +1121,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>47</v>
       </c>
@@ -1133,7 +1132,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
@@ -1144,7 +1143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>51</v>
       </c>
@@ -1155,7 +1154,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>54</v>
       </c>
@@ -1166,7 +1165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>56</v>
       </c>
@@ -1177,7 +1176,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>58</v>
       </c>
@@ -1188,7 +1187,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>60</v>
       </c>
@@ -1199,7 +1198,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>62</v>
       </c>
@@ -1210,7 +1209,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>64</v>
       </c>
@@ -1221,7 +1220,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>66</v>
       </c>
@@ -1232,7 +1231,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>68</v>
       </c>
@@ -1243,7 +1242,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>70</v>
       </c>
@@ -1254,7 +1253,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>72</v>
       </c>
@@ -1265,7 +1264,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>74</v>
       </c>
@@ -1276,7 +1275,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>76</v>
       </c>
@@ -1287,7 +1286,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>78</v>
       </c>
@@ -1298,7 +1297,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>80</v>
       </c>
@@ -1309,7 +1308,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>83</v>
       </c>
@@ -1320,7 +1319,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>85</v>
       </c>
@@ -1331,7 +1330,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>87</v>
       </c>
@@ -1342,7 +1341,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>90</v>
       </c>
@@ -1353,7 +1352,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>92</v>
       </c>
@@ -1364,7 +1363,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>94</v>
       </c>
@@ -1375,7 +1374,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>97</v>
       </c>
@@ -1386,7 +1385,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>99</v>
       </c>
@@ -1397,7 +1396,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>101</v>
       </c>
@@ -1408,7 +1407,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>103</v>
       </c>
@@ -1419,7 +1418,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>105</v>
       </c>
@@ -1430,7 +1429,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>107</v>
       </c>
@@ -1441,7 +1440,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>109</v>
       </c>
@@ -1452,7 +1451,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>111</v>
       </c>
@@ -1463,7 +1462,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>113</v>
       </c>
@@ -1474,7 +1473,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>115</v>
       </c>
@@ -1485,7 +1484,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>117</v>
       </c>
@@ -1496,7 +1495,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>119</v>
       </c>
@@ -1507,7 +1506,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>121</v>
       </c>
@@ -1518,7 +1517,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>123</v>
       </c>
@@ -1529,7 +1528,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>125</v>
       </c>
@@ -1540,7 +1539,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>127</v>
       </c>
@@ -1551,7 +1550,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>129</v>
       </c>
@@ -1562,7 +1561,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>131</v>
       </c>
@@ -1573,7 +1572,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>133</v>
       </c>
@@ -1584,7 +1583,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>135</v>
       </c>
@@ -1595,7 +1594,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>137</v>
       </c>
@@ -1606,7 +1605,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>139</v>
       </c>
@@ -1617,7 +1616,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>141</v>
       </c>
@@ -1628,7 +1627,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>143</v>
       </c>
@@ -1639,7 +1638,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>145</v>
       </c>
@@ -1650,7 +1649,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>34</v>
       </c>
@@ -1661,7 +1660,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>148</v>
       </c>
@@ -1672,7 +1671,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>150</v>
       </c>
@@ -1683,7 +1682,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>152</v>
       </c>
@@ -1694,7 +1693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>154</v>
       </c>
@@ -1705,7 +1704,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>156</v>
       </c>
@@ -1716,7 +1715,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>158</v>
       </c>
@@ -1727,7 +1726,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>160</v>
       </c>
@@ -1738,7 +1737,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>162</v>
       </c>
@@ -1749,7 +1748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>164</v>
       </c>
@@ -1760,7 +1759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>166</v>
       </c>
@@ -1771,7 +1770,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>168</v>
       </c>
@@ -1782,7 +1781,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>170</v>
       </c>
@@ -1793,7 +1792,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>172</v>
       </c>
@@ -1805,13 +1804,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C81" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Gestión de Asesoría Jurídica / Dirección de Asesoría Jurídica"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:C81" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>